<commit_message>
feat: v0.3 - replicate-weights variance engine
- rep_weights role in lst_data(): explicit columns or prefix expansion
  (W_FSTR -> W_FSTR1..R, PISA style), rep_method fay/brr/jk1/jk2 with
  fay_k, validated with friendly errors
- compute_stat_rep(): sampling variance = factor * sum((est_r - est)^2)
  applied uniformly to all statistics via est_stat() (estimates proven
  identical to compute_stat); measurement variance from individual IRT
  SEs still added orthogonally
- wired through lst_table (meta records variance = replicate:<method>),
  item p-values, YAML/JSON config, JSON Schema, Excel template and
  lst_run column pruning (csv header peek for prefix expansion)
- Monte Carlo cluster test: JK1 SE 0.0702 vs empirical 0.0722 while
  linearized formula gives 0.0339 (design effect ~4x)
</commit_message>
<xml_diff>
--- a/inst/templates/config-template.xlsx
+++ b/inst/templates/config-template.xlsx
@@ -571,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -678,6 +678,45 @@
       <c r="C6" t="inlineStr">
         <is>
           <t>观察得分,可留空</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>复制权重列</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>如 W_FSTR(前缀,自动展开为W_FSTR1..R)或逗号分隔列名;不用可留空</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>复制权重方法</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>fay(PISA)/brr/jk1/jk2(TIMSS);用了复制权重必填</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Fay系数</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>仅 fay 方法需要,默认 0.5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: v0.4 - plausible values (Rubin) engine and HTML reports
- pv role in lst_data(): PV#MATH template expansion, pv_sampling
  first/average conventions; all statistics on PV dimensions use Rubin
  combination (total variance = sampling U + (1+1/M)B imputation),
  composing with replicate weights for the full PISA variance recipe
  (meta: variance = rubin+replicate:fay)
- method = prob rejected on PV dimensions with explanatory guidance
- dependency-free lst_to_html(): styled standalone report with pivot
  tables, rule-based interpretation and variance-method footnote;
  html output wired into lst_run(), schema and Excel template
  (dimension sheet gains a PV column, output sheet gains HTML)
- Monte Carlo: Rubin total-variance coverage 0.99, PV hard-classified
  level proportions calibrated to the latent distribution
- fix: resolve_stat_var now includes pv dimension names; lst_run column
  pruning no longer passes pv dimension names to fread
</commit_message>
<xml_diff>
--- a/inst/templates/config-template.xlsx
+++ b/inst/templates/config-template.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -483,78 +483,85 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2.「能力维度」:每行一个能力维度(维度名、能力值列、标准误列)。没有能力值可留空。</t>
+          <t>2.「能力维度」:每行一个能力维度。有点估计填能力值列+标准误列;</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3.「统计表」:每行定义一个统计量;同一「表名」的行会合成一张透视表。</t>
+          <t xml:space="preserve">   有 plausible values 填 PV列(如 PV#READ,# 代表编号,自动展开为 PV1READ..)。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">   统计量可选: st_mean(均值) st_sd(标准差) st_prop_above(超阈值占比)</t>
+          <t>3.「统计表」:每行定义一个统计量;同一「表名」的行会合成一张透视表。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">   st_level_prop(等级占比) st_quantile(分位数) st_count(人数) st_wcount(加权人数)</t>
+          <t xml:space="preserve">   统计量可选: st_mean(均值) st_sd(标准差) st_prop_above(超阈值占比)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   st_pvalue(题目正答率) st_option_dist(选项分布)</t>
+          <t xml:space="preserve">   st_level_prop(等级占比) st_quantile(分位数) st_count(人数) st_wcount(加权人数)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">   方法: hard(硬分类) 或 prob(概率化,利用每人的标准误,推荐)</t>
+          <t xml:space="preserve">   st_pvalue(题目正答率) st_option_dist(选项分布)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   校正: 留空(EAP能力值) 或 latent(WLE/ML能力值)</t>
+          <t xml:space="preserve">   方法: hard(硬分类) 或 prob(概率化,利用每人的标准误,推荐)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">   等级分数线格式: 低=-Inf,中=0,高=1(等级名=下界,逗号分隔)</t>
+          <t xml:space="preserve">   校正: 留空(EAP能力值) 或 latent(WLE/ML能力值)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>4.「输出」:填希望生成的 Excel / JSON 文件路径。</t>
+          <t xml:space="preserve">   等级分数线格式: 低=-Inf,中=0,高=1(等级名=下界,逗号分隔)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>4.「输出」:填希望生成的 Excel / JSON 文件路径。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>5. 在 R 中运行: LISTR::lst_run("本文件路径.xlsx")</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>注意:不要删除或重命名工作表;灰色斜体行是示例,可直接修改。</t>
         </is>
@@ -731,12 +738,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -755,6 +763,11 @@
           <t>标准误列</t>
         </is>
       </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>PV列</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -770,6 +783,21 @@
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>se_math</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr"/>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>PV#READ</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1119,6 +1147,23 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HTML输出路径</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>results.html</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>留空则不输出 HTML 报告</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>